<commit_message>
created relationship diagram for PBI semantic model
</commit_message>
<xml_diff>
--- a/docs/20_Data_Dictionary.xlsx
+++ b/docs/20_Data_Dictionary.xlsx
@@ -5224,9 +5224,14 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>(as Volume Stress Sensitivity, but returning)
-DIVIDE ( Cov, SQRT ( SUMX ( Known, ( [@x] - MeanX ) ^ 2 ) )
-            * SQRT ( SUMX ( Known, ( [@y] - MeanY ) ^ 2 ) ) )</t>
+          <t>VAR Points = ADDCOLUMNS ( CALCULATETABLE ( VALUES ( DimDate[DateKey] ), ALLSELECTED ( DimDate ) ),
+    "@x", [Consumer Stress Index], "@y", [Total Cases YoY %] )
+VAR Known = FILTER ( Points, NOT ISBLANK ( [@x] ) &amp;&amp; NOT ISBLANK ( [@y] ) )
+VAR MeanX = AVERAGEX ( Known, [@x] )
+VAR MeanY = AVERAGEX ( Known, [@y] )
+VAR Cov = SUMX ( Known, ( [@x] - MeanX ) * ( [@y] - MeanY ) )
+RETURN DIVIDE ( Cov, SQRT ( SUMX ( Known, ( [@x] - MeanX ) ^ 2 ) )
+              * SQRT ( SUMX ( Known, ( [@y] - MeanY ) ^ 2 ) ) )</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
@@ -5236,7 +5241,7 @@
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>Pearson r on the same points. Reported beside the slope so a reader can see how much of the relationship the slope explains.</t>
+          <t>Pearson r on the same points as Volume Stress Sensitivity. Reported beside the slope so a reader can see how much of the relationship the slope explains. Written out in full rather than as a note, because a measure cannot inherit another measure's variables.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
doc cleanup after changes
</commit_message>
<xml_diff>
--- a/docs/20_Data_Dictionary.xlsx
+++ b/docs/20_Data_Dictionary.xlsx
@@ -907,7 +907,7 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>NAICS kind-of-business code. Nineteen codes are requested; 44X72 and 44000 are aggregates and are excluded from share denominators.</t>
+          <t>NAICS kind-of-business code. The published set is discovered at refresh rather than requested as a fixed list — 21 codes on 22 September 2026. Five are aggregates and are excluded from share denominators: 44X72, 44000, 44W72, 44Y72 and 44Z72.</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>TRUE for 44X72 and 44000 only. Excluded from share denominators so the aggregate is not double-counted.</t>
+          <t>TRUE for every total and “excluding” aggregate — 44X72, 44000, 44W72, 44Y72 and 44Z72 on the 22 September 2026 set. Excluded from share denominators so the aggregate is not double-counted.</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>TRUE for 44X72 and 44000. Share of Total Retail % returns blank for aggregates so they cannot appear as a share of themselves.</t>
+          <t>TRUE for every total and “excluding” aggregate — 44X72, 44000, 44W72, 44Y72 and 44Z72 on the 22 September 2026 set. Share of Total Retail % returns blank for aggregates so they cannot appear as a share of themselves.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
updating documenatation after fixing missing code information
</commit_message>
<xml_diff>
--- a/docs/20_Data_Dictionary.xlsx
+++ b/docs/20_Data_Dictionary.xlsx
@@ -1853,7 +1853,7 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>21</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>≈ 2,180</t>
+          <t>≈ 2,940</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">

</xml_diff>